<commit_message>
À propos : coordonnées Commercial/SAV, devis à champs obligatoires, accents réactifs
- À propos : ajoute les numéros Commercial (+213.770.08.54.53) et SAV
  (+213.770.74.72.50) dans le bloc Téléphone / Fax.
- Devis (ModalDevis) : Organisme, Nom, Téléphone et Email rendus
  obligatoires (indicateur * + validation) ; clé de liste panier fiabilisée.
- Réactifs (données) : corrige accents et espacement du champ
  conditionnement (« contrôle et calibrant inclus ») sur les kits combo.
- Rapport des changements (xlsx) mis à jour.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rapport_changes_biointeraction.xlsx
+++ b/rapport_changes_biointeraction.xlsx
@@ -107,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -140,6 +140,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -507,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -749,6 +752,102 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>A propos</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>app/a-propos/page.tsx</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Ajout</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Ajout des numeros Commercial (+213.770.08.54.53) et SAV (+213.770.74.72.50) dans le bloc Telephone / Fax.</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Devis</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>src/components/ModalDevis.tsx</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Amelioration</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Champs Organisme, Nom, Telephone et Email rendus obligatoires (indicateur * + validation). Cle de liste panier fiabilisee.</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Catalogue reactifs (donnees)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>src/data/products-reactifs.ts</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Correction</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Correction d'accents et d'espacement du champ conditionnement (« controle et calibrant inclus ») sur les kits combo.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Rapport : consigne la traduction FR de l'article CytoBead ANA 2
Ajoute une ligne « Traduction » documentant la traduction française du
corps de l'article blog « CytoBead ANA 2 » (Firestore), avec préservation
de la structure et correction des liens https://https://.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rapport_changes_biointeraction.xlsx
+++ b/rapport_changes_biointeraction.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,6 +55,11 @@
     <font>
       <b val="1"/>
       <color rgb="0015803D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000082A0"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -107,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -143,6 +148,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -510,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -848,6 +856,38 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Blog (Firestore)</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Article « CytoBead ANA 2 » — Firestore, collection articles (doc Cm3oq5GF9gh80SOzgCJh)</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Traduction</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Traduction FR du corps de l'article « Une nouvelle etude met en lumiere le pouvoir diagnostique de CytoBead ANA 2 » (blocs anglais traduits ; titre, chapo, images, tableaux, liens et noms de produits preserves ; 2 liens https://https:// corriges).</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>En ligne / verifie</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Securite: durcissements (anti-tabnabbing, emailVerified) + audit consigne
- sanitize.ts: rel=noopener noreferrer force sur les liens target=_blank du blog.

- send-devis: refus (403) si l'email du compte n'est pas verifie.

- package-lock: dedup uuid + bump mineur firestore (npm audit fix).

- rapport_changes: audit de securite et correctifs consignes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rapport_changes_biointeraction.xlsx
+++ b/rapport_changes_biointeraction.xlsx
@@ -112,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -151,6 +151,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -518,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -888,6 +891,70 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Securite — Audit</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>(transverse : routes API, regles Firestore/Storage, next.config, lib)</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Audit de securite complet (authn/authz, XSS, injection, secrets, dependances, en-tetes HTTP, SSRF, CSRF) + tests dynamiques en production (en-tetes actifs, gate CSRF renvoie 400). Aucune faille critique ni elevee. Quelques durcissements moyens/faibles identifies.</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Realise</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Securite — Durcissement</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>src/lib/sanitize.ts, app/api/send-devis/route.ts, package-lock.json</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Correction</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Liens blog : rel="noopener noreferrer" force sur target=_blank (anti-tabnabbing). Route devis : verification emailVerified (403 si non verifie). Dependances : npm audit fix (dedup uuid, bump mineur firestore). 10 vulns moderees restantes necessitent une montee majeure firebase-admin/next.</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>tsc OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: permissions locales + rapport (investigation vulns dependances)
- .claude/settings.local.json : permissions de session.

- rapport_changes : investigation des 10 vulns moderees consignee (non corrigeables sans rupture, baseline saine conservee).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rapport_changes_biointeraction.xlsx
+++ b/rapport_changes_biointeraction.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -955,6 +955,38 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Securite — Dependances</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>package.json / package-lock.json (investigation, sans changement net)</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Investigation des 10 vulnerabilites moderees (npm audit). Non corrigeables sans rupture : le postcss vulnerable est bundle dans Next (le seul fix npm = downgrade absurde) ; chaine firebase-admin transitive (la v14 testee ne corrige que 2/10 et exige Node&gt;=22, risque Vercel). Revenu a la baseline saine sous filet de sauvegarde git ; advisories acceptees (faible exploitabilite, surveillance via npm audit).</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Aucune rupture</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
rapport: firebase-admin@14 applique (10 -> 8 vulns)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rapport_changes_biointeraction.xlsx
+++ b/rapport_changes_biointeraction.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -987,6 +987,38 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Securite — Dependances</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>package.json, package-lock.json</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Correction</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>firebase-admin 13 -&gt; 14 applique (Vercel confirme en Node 26.3.0). Elimine 2 des vulns transitives (10 -&gt; 8). engines.node &gt;=22 ajoute comme garde. Build compilation/TypeScript OK. Les 8 restantes (postcss bundle dans Next + chaine google-gax/gaxios/uuid en amont) restent non corrigeables sans rupture.</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Build OK / pousse</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Catalogue: ajoute 2 analyseurs ERBA + categorie Immunologie
Ajout des equipements manquants ERBA LISA SCAN (ref 52000121, lecteur ELISA) et ERBA LISA WASH (ref 52000131, laveur ELISA) dans une nouvelle categorie Immunologie.

- products-equip.ts : section Immunologie + 2 produits
- fiches-equipements.ts : brochure commune LisaScan/LisaWash
- EquipementsContent.tsx + EquipementsLanding.tsx : filtre, carte categorie et icone microplaque ELISA
- Navbar.tsx : entree menu deroulant Equipements
- images telechargees depuis erbalachema.com
- rapport_changes_biointeraction.xlsx mis a jour

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rapport_changes_biointeraction.xlsx
+++ b/rapport_changes_biointeraction.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Changements" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -26,40 +25,49 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001D4ED8"/>
+      <color rgb="FF1D4ED8"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00B30C2F"/>
+      <color rgb="FFB30C2F"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="007E22CE"/>
+      <color rgb="FF7E22CE"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="0015803D"/>
+      <color rgb="FF15803D"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000082A0"/>
+      <color rgb="FF0082A0"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -72,17 +80,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B1F1D"/>
+        <fgColor rgb="FF1B1F1D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0029A864"/>
+        <fgColor rgb="FF29A864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDF8F1"/>
+        <fgColor rgb="FFEDF8F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -96,69 +104,71 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D8D8D2"/>
+        <color rgb="FFD8D8D2"/>
       </left>
       <right style="thin">
-        <color rgb="00D8D8D2"/>
+        <color rgb="FFD8D8D2"/>
       </right>
       <top style="thin">
-        <color rgb="00D8D8D2"/>
+        <color rgb="FFD8D8D2"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D8D8D2"/>
+        <color rgb="FFD8D8D2"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -519,503 +529,535 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="66" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" style="15" min="1" max="1"/>
+    <col width="22" customWidth="1" style="15" min="2" max="2"/>
+    <col width="46" customWidth="1" style="15" min="3" max="3"/>
+    <col width="14" customWidth="1" style="15" min="4" max="4"/>
+    <col width="66" customWidth="1" style="15" min="5" max="5"/>
+    <col width="18" customWidth="1" style="15" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="27.95" customHeight="1" s="15">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>BioInteraction — Rapport des modifications du site web</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="21.95" customHeight="1" s="15">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Zone / Page</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Fichier(s)</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>Validation</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+    <row r="3" ht="25.5" customHeight="1" s="15">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Accueil</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>src/components/homepage/VoirNosProduitsCTA.tsx (nouveau), app/page.tsx</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Ajout</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Le bouton « Voir Nos Produits » du Hero ouvre un popup de choix Equipements / Reactifs ; chaque choix mene a la page catalogue correspondante.</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>tsc OK / build OK</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
+    <row r="4" ht="25.5" customHeight="1" s="15">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Partenaires</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>app/partenaires/page.tsx</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Localisation d'ERBA Mannheim corrigee : Allemagne -&gt; Republique Tcheque (drapeau et libelle pays).</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>tsc OK</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
+    <row r="5" ht="25.5" customHeight="1" s="15">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Accueil - Guide FAQ</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>src/components/homepage/FaqAssistant.tsx, src/data/faq.ts</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Amelioration</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Boutons d'action dans les reponses (devis / contact / catalogue / partenaires), nouvel item FAQ « Produits », suggestion rapide « Voir nos produits ».</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>tsc OK</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
+    <row r="6" ht="38.25" customHeight="1" s="15">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Guide intelligent</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>src/components/SmartGuide.tsx, src/components/catalogue/CatalogueClient.tsx</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Dans les resultats du guide, cliquer un produit ouvre desormais sa fiche dediee (parametre d'URL ?ref=) au lieu de la categorie entiere. Toute la carte est cliquable.</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>tsc OK</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+    <row r="7" ht="51" customHeight="1" s="15">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Catalogue equipements</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>src/components/catalogue/CatalogueClient.tsx</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Bouton « Voir les reactifs compatibles » : navigation vers la section de reactifs dediee de chaque analyseur (cat + section) au lieu d'une recherche texte fragile qui ramenait des faux positifs (ex. EC 90 : 9 cartouches exactes au lieu de 17 melangees).</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Tests data OK</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
+    <row r="8" ht="38.25" customHeight="1" s="15">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Qualite / Tests</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>(transverse)</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Verification</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Batterie de tests d'integrite : refs SmartGuide, COMPAT_MAP (17 analyseurs couverts), 436 images presentes, hrefs valides, doublons reactifs confirmes intentionnels. Aucun bug reel detecte.</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
+    <row r="9" ht="25.5" customHeight="1" s="15">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>A propos</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>app/a-propos/page.tsx</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Ajout</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Ajout des numeros Commercial (+213.770.08.54.53) et SAV (+213.770.74.72.50) dans le bloc Telephone / Fax.</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
+    <row r="10" ht="25.5" customHeight="1" s="15">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Devis</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>src/components/ModalDevis.tsx</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>Amelioration</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Champs Organisme, Nom, Telephone et Email rendus obligatoires (indicateur * + validation). Cle de liste panier fiabilisee.</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+    <row r="11" ht="25.5" customHeight="1" s="15">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Catalogue reactifs (donnees)</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>src/data/products-reactifs.ts</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Correction d'accents et d'espacement du champ conditionnement (« controle et calibrant inclus ») sur les kits combo.</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
+    <row r="12" ht="51" customHeight="1" s="15">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Blog (Firestore)</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Article « CytoBead ANA 2 » — Firestore, collection articles (doc Cm3oq5GF9gh80SOzgCJh)</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Traduction</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Traduction FR du corps de l'article « Une nouvelle etude met en lumiere le pouvoir diagnostique de CytoBead ANA 2 » (blocs anglais traduits ; titre, chapo, images, tableaux, liens et noms de produits preserves ; 2 liens https://https:// corriges).</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>En ligne / verifie</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
+    <row r="13" ht="51" customHeight="1" s="15">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Securite — Audit</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>(transverse : routes API, regles Firestore/Storage, next.config, lib)</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>Verification</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Audit de securite complet (authn/authz, XSS, injection, secrets, dependances, en-tetes HTTP, SSRF, CSRF) + tests dynamiques en production (en-tetes actifs, gate CSRF renvoie 400). Aucune faille critique ni elevee. Quelques durcissements moyens/faibles identifies.</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Realise</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
+    <row r="14" ht="51" customHeight="1" s="15">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Securite — Durcissement</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>src/lib/sanitize.ts, app/api/send-devis/route.ts, package-lock.json</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Liens blog : rel="noopener noreferrer" force sur target=_blank (anti-tabnabbing). Route devis : verification emailVerified (403 si non verifie). Dependances : npm audit fix (dedup uuid, bump mineur firestore). 10 vulns moderees restantes necessitent une montee majeure firebase-admin/next.</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>tsc OK</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
+    <row r="15" ht="76.5" customHeight="1" s="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Securite — Dependances</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>package.json / package-lock.json (investigation, sans changement net)</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Verification</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Investigation des 10 vulnerabilites moderees (npm audit). Non corrigeables sans rupture : le postcss vulnerable est bundle dans Next (le seul fix npm = downgrade absurde) ; chaine firebase-admin transitive (la v14 testee ne corrige que 2/10 et exige Node&gt;=22, risque Vercel). Revenu a la baseline saine sous filet de sauvegarde git ; advisories acceptees (faible exploitabilite, surveillance via npm audit).</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Aucune rupture</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
+    <row r="16" ht="51" customHeight="1" s="15">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Securite — Dependances</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>package.json, package-lock.json</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>firebase-admin 13 -&gt; 14 applique (Vercel confirme en Node 26.3.0). Elimine 2 des vulns transitives (10 -&gt; 8). engines.node &gt;=22 ajoute comme garde. Build compilation/TypeScript OK. Les 8 restantes (postcss bundle dans Next + chaine google-gax/gaxios/uuid en amont) restent non corrigeables sans rupture.</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Deploye en prod / vert</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Catalogue equipements / Immunologie</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>src/data/products-equip.ts, src/data/fiches-equipements.ts, src/components/catalogue/EquipementsContent.tsx, src/components/catalogue/EquipementsLanding.tsx, src/components/Navbar.tsx, public/images/equipements/</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Ajout</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Ajout de 2 analyseurs ERBA manquants au catalogue et creation de la categorie Immunologie : ERBA LISA SCAN (ref 52000121, lecteur ELISA) et ERBA LISA WASH (ref 52000131, laveur ELISA). Section Immunologie ajoutee (data, landing avec icone microplaque, filtre, menu Navbar). Fiches/brochure commune LisaScan-LisaWash. Images telechargees depuis erbalachema.com.</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>tsc OK / preview 200 (landing, ?cat=immunologie, ?all=1) / images 200</t>
         </is>
       </c>
     </row>
@@ -1023,6 +1065,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="80" fitToHeight="0" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Catalogue: corrige conditionnement ELISA + lie reactifs LISA SCAN
- products-equip.ts : conditionnement reel des 2 analyseurs (LISA SCAN = 100 protocoles ELISA programmables ; LISA WASH = 50 protocoles de lavage)
- CatalogueClient.tsx : COMPAT_MAP lie ERBA LISA SCAN (52000121) a la section reactifs Auto-Immunite -ELISA Manuel (39 reactifs Generic Assays)
- rapport_changes_biointeraction.xlsx mis a jour

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rapport_changes_biointeraction.xlsx
+++ b/rapport_changes_biointeraction.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="15" min="1" max="1"/>
@@ -1061,6 +1061,38 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Catalogue equipements / Immunologie</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>src/data/products-equip.ts, src/components/catalogue/CatalogueClient.tsx</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Correction</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Conditionnement reel des 2 analyseurs ELISA corrige : ERBA LISA SCAN = 100 protocoles de test ELISA programmables par l utilisateur ; ERBA LISA WASH = 50 protocoles de lavage definis par l utilisateur. Liaison reactifs ajoutee : bouton Voir les reactifs compatibles d ERBA LISA SCAN pointe vers la section Auto-Immunite -ELISA Manuel (39 reactifs Generic Assays deja presents).</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>tsc OK / preview 200 (page reactifs compatibles affiche les 39 ELISA Manuel)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Guide intelligent: ajoute la categorie Immunologie (LISA SCAN + WASH)
Etape equip-domaine du SmartGuide : nouvelle branche Immunologie proposant ERBA LISA SCAN (52000121) et ERBA LISA WASH (52000131), oubliee lors de l'ajout initial des 2 analyseurs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rapport_changes_biointeraction.xlsx
+++ b/rapport_changes_biointeraction.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="15" min="1" max="1"/>
@@ -1093,6 +1093,38 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Guide intelligent</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>src/components/SmartGuide.tsx</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Ajout</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Ajout de la categorie Immunologie dans l arbre du guide intelligent (etape equip-domaine) : propose ERBA LISA SCAN (52000121) et ERBA LISA WASH (52000131). Oubli de la mise a jour lors de l ajout initial des 2 analyseurs.</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>tsc OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Catalogue reactifs : retrait de 2 references ERBA + image CytoBead ANA 2
- Suppression des reactifs ERBA Thrombin Time (EHL00007) et Erba Chrom
  Protein C (EHL00009), avec leurs entrees de fiches techniques (IFU)
- CytoBead ANA 2 (ref 8220) : image alignee sur CytoBead ANA
  (ga-ifi-hep2.jpg -> ga-cytobead-slides.png)
- Rapport des changements mis a jour

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rapport_changes_biointeraction.xlsx
+++ b/rapport_changes_biointeraction.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="15" min="1" max="1"/>
@@ -1413,6 +1413,70 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Catalogue - Reactifs Hemostase</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>src/data/products-reactifs.ts, src/data/fiches-techniques.ts</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Suppression</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Retrait des reactifs ERBA Thrombin Time (EHL00007) et Erba Chrom Protein C (EHL00009), ainsi que leurs entrees de fiches techniques (notices IFU).</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>tsc OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Catalogue - Reactifs Auto-Immunite</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>src/data/products-reactifs.ts</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Correction</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Image de CytoBead ANA 2 (ref 8220) alignee sur celle de CytoBead ANA : ga-ifi-hep2.jpg -&gt; ga-cytobead-slides.png.</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>tsc OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Partenaires & catalogue : descriptions HOB/LDBIO + renommage sous-categories
- Partenaires : nouvelles descriptions HOB Biotech (Suzhou, 2007, collaboration 2023) et LDBIO Diagnostics (partenaire historique).
- Catalogue reactifs Biochimie : "Reactifs Systeme Ferme" -> "Reactifs Adaptes" ; "Reactifs Systeme Ouvert" -> "Reactifs Systeme Ouvert / Manuels".
- Rapport des changements mis a jour.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rapport_changes_biointeraction.xlsx
+++ b/rapport_changes_biointeraction.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="15" min="1" max="1"/>
@@ -1445,7 +1445,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" s="15">
       <c r="A30" s="5" t="inlineStr">
         <is>
           <t>2026-06-11</t>
@@ -1474,6 +1474,70 @@
       <c r="F30" s="6" t="inlineStr">
         <is>
           <t>tsc OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" s="15">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Partenaires</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>app/partenaires/page.tsx</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Amelioration</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>Descriptions partenaires reecrites : HOB Biotech (entreprise biotech chinoise fondee en 2007 a Suzhou, allergologie et auto-immunite ; collaboration depuis 2023) et LDBIO Diagnostics (partenaire historique, expertise parasitologie/mycologie).</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>preview OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" s="15">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Catalogue - Reactifs Biochimie</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>src/components/catalogue/ReactifsSubcategoryLanding.tsx</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Amelioration</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Renommage des libelles de sous-categories (SECTION_DISPLAY) : Reactifs Systeme Ferme -&gt; Reactifs Adaptes ; Reactifs Systeme Ouvert -&gt; Reactifs Systeme Ouvert / Manuels. Cles brutes (identifiants) inchangees.</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>preview OK</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Blog editeur : suppression de l anti-pattern react-hooks/refs (cles en state)
L editeur de liste enrichie geraient les cles React via une ref lue et mutee pendant le rendu (react-hooks/refs). Migration vers un state useState avec realignement pendant le rendu + mutations positionnelles dans les handlers. Comportement preserve. Rapport mis a jour.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rapport_changes_biointeraction.xlsx
+++ b/rapport_changes_biointeraction.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="15" min="1" max="1"/>
@@ -1541,6 +1541,38 @@
         </is>
       </c>
     </row>
+    <row r="33" s="15">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Blog - Editeur (Nouvel article)</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>app/blog/new/page.tsx</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Correction</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Editeur de liste enrichie : suppression de l anti-pattern react-hooks/refs (ref stableKeys lue/mutee pendant le rendu). Les cles React stables sont desormais gerees en state (useState) avec realignement pendant le rendu et mutations positionnelles dans les handlers. Comportement preserve (focus contentEditable stable).</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>tsc OK / lint refs OK / /blog/new 200</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>